<commit_message>
Move to Completed | Edit Distro Lists
</commit_message>
<xml_diff>
--- a/Reference Data/XLSX Workbooks/Internal CC Lists.xlsx
+++ b/Reference Data/XLSX Workbooks/Internal CC Lists.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arch Aerial WS 01\Documents\Data Team\Steven\Dailies Email Templates\Reference Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arch Aerial WS 01\Documents\Data Team\Steven\Customer Email Builder\Reference Data\XLSX Workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D45FE5-C7A2-4CCA-8CC9-C1C0222DFB70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF5B59A6-F2C3-4462-9CEE-AD6AF9F2ACC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-16440" windowWidth="38640" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Steven" sheetId="1" r:id="rId1"/>
-    <sheet name="Doug" sheetId="2" r:id="rId2"/>
+    <sheet name="Doug" sheetId="1" r:id="rId1"/>
+    <sheet name="Steven" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="10">
   <si>
     <t>Commercial Construction</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>dsimpson@archaerial.com</t>
-  </si>
-  <si>
-    <t>msweisthal@archaerial.com</t>
   </si>
   <si>
     <t>smclaren@archaerial.com</t>
@@ -425,12 +422,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="28.28515625" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -482,14 +475,9 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
         <v>9</v>
       </c>
     </row>
@@ -499,12 +487,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{326773E8-2C0F-4737-B0F1-2FBA241AAD70}">
-  <dimension ref="A1:B8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.28515625" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" customWidth="1"/>
+    <col min="1" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -557,22 +544,13 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A7" r:id="rId1" xr:uid="{9C0D5212-21C3-440E-9FFF-9B17F4AB58EC}"/>
-    <hyperlink ref="B7" r:id="rId2" xr:uid="{489597AE-1961-4D9E-9D53-DC6A60540491}"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Additional GFT template formatting optimization | EML Signature script stripper revamp
</commit_message>
<xml_diff>
--- a/Reference Data/XLSX Workbooks/Internal CC Lists.xlsx
+++ b/Reference Data/XLSX Workbooks/Internal CC Lists.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doug" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steven" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__pycache__" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -663,4 +664,30 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Commercial Construction</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>